<commit_message>
implemented muster page api integration
</commit_message>
<xml_diff>
--- a/src/main/resources/timesheet_template.xlsx
+++ b/src/main/resources/timesheet_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/manishabharti/Sandbox/varista-service/src/main/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Sandbox\Varista\varista-service\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E25545-2E2A-D04F-B523-EAD28273346E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F6A3643-4FCA-4060-80A9-7B778AA43E20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="16440" windowHeight="28320" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Muster " sheetId="2" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master Muster '!$A$8:$AT$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Wage'!$A$9:$AE$9</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Master Muster '!$A$1:$AT$15</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Master Wage'!$A$1:$AE$16</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Master Wage'!$A$1:$AE$45</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Master Muster '!$1:$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Master Wage'!$1:$9</definedName>
   </definedNames>
@@ -36,15 +36,17 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="62">
   <si>
     <t xml:space="preserve">Muster Register Form II </t>
   </si>
@@ -124,39 +126,6 @@
     <t>1 Hr</t>
   </si>
   <si>
-    <t>Supervisor</t>
-  </si>
-  <si>
-    <t>Welder</t>
-  </si>
-  <si>
-    <t>Tag Welder</t>
-  </si>
-  <si>
-    <t>RAM KUMAR</t>
-  </si>
-  <si>
-    <t>BIKASH KUMAR SINGH</t>
-  </si>
-  <si>
-    <t>VIJAY SAHU</t>
-  </si>
-  <si>
-    <t>BRIJKISHOR YADAV</t>
-  </si>
-  <si>
-    <t>Rohit Vishwakarma</t>
-  </si>
-  <si>
-    <t>ANKIT KUMAR GIRI</t>
-  </si>
-  <si>
-    <t>LE24M354</t>
-  </si>
-  <si>
-    <t>Varista Industrial Solutions</t>
-  </si>
-  <si>
     <t xml:space="preserve">Wage Sheet </t>
   </si>
   <si>
@@ -262,31 +231,8 @@
     <t>REMARK</t>
   </si>
   <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>BABAN SINGH</t>
-  </si>
-  <si>
-    <t>HARIOM</t>
-  </si>
-  <si>
-    <t>AYODHYA CHAUHAN</t>
-  </si>
-  <si>
-    <t>RAM ADHAR</t>
-  </si>
-  <si>
-    <t>CHHATHU YADAV</t>
-  </si>
-  <si>
-    <t>ANIL GIRI</t>
-  </si>
-  <si>
-    <t>SSK</t>
-  </si>
-  <si>
-    <t>SK</t>
+    <t>Name and Address of Principle Employer  :
+JSW, Pen, Raigardh, Maharashtra</t>
   </si>
 </sst>
 </file>
@@ -296,7 +242,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\/mm\/yyyy"/>
   </numFmts>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -387,84 +333,10 @@
     </font>
     <font>
       <b/>
-      <sz val="24"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="22"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="24"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="24"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="24"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="28"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="20"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="28"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="28"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="36"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri Light"/>
-      <family val="2"/>
-      <scheme val="major"/>
     </font>
   </fonts>
   <fills count="4">
@@ -532,7 +404,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="97">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -660,114 +532,70 @@
     <xf numFmtId="1" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="18" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="8" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="1" fontId="19" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="13" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="21" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="22" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="21" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="21" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="23" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="1" fontId="22" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="19" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="24" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -807,92 +635,18 @@
     </xf>
     <xf numFmtId="17" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="62">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="54">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1713,179 +1467,179 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AT15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.5" style="39" customWidth="1"/>
-    <col min="2" max="2" width="30.5" style="39" customWidth="1"/>
+    <col min="1" max="1" width="12.42578125" style="39" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" style="39" customWidth="1"/>
     <col min="3" max="3" width="35" style="39" customWidth="1"/>
-    <col min="4" max="4" width="46.5" style="40" customWidth="1"/>
-    <col min="5" max="5" width="24.33203125" style="41" customWidth="1"/>
-    <col min="6" max="6" width="21.6640625" style="42" customWidth="1"/>
-    <col min="7" max="7" width="21.6640625" style="43" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" style="39" customWidth="1"/>
+    <col min="4" max="4" width="46.42578125" style="40" customWidth="1"/>
+    <col min="5" max="5" width="24.28515625" style="41" customWidth="1"/>
+    <col min="6" max="6" width="21.7109375" style="42" customWidth="1"/>
+    <col min="7" max="7" width="21.7109375" style="43" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.85546875" style="39" customWidth="1"/>
     <col min="9" max="9" width="7" style="39" customWidth="1"/>
-    <col min="10" max="32" width="5.33203125" style="39" customWidth="1"/>
-    <col min="33" max="40" width="5.5" style="39" customWidth="1"/>
-    <col min="41" max="41" width="10.83203125" style="39" customWidth="1"/>
-    <col min="42" max="42" width="9.5" style="39" customWidth="1"/>
+    <col min="10" max="32" width="5.28515625" style="39" customWidth="1"/>
+    <col min="33" max="40" width="5.42578125" style="39" customWidth="1"/>
+    <col min="41" max="41" width="10.85546875" style="39" customWidth="1"/>
+    <col min="42" max="42" width="9.42578125" style="39" customWidth="1"/>
     <col min="43" max="43" width="9" style="39" customWidth="1"/>
-    <col min="44" max="44" width="20.1640625" style="39" customWidth="1"/>
+    <col min="44" max="44" width="20.140625" style="39" customWidth="1"/>
     <col min="45" max="45" width="43" style="41" customWidth="1"/>
-    <col min="46" max="46" width="24.5" style="39" bestFit="1" customWidth="1"/>
-    <col min="47" max="16384" width="9.1640625" style="39"/>
+    <col min="46" max="46" width="24.42578125" style="39" bestFit="1" customWidth="1"/>
+    <col min="47" max="16384" width="9.140625" style="39"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:46" s="3" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="86" t="s">
+    <row r="1" spans="1:46" s="3" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="70" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="86"/>
-      <c r="C1" s="86"/>
-      <c r="D1" s="87"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="86"/>
-      <c r="G1" s="86"/>
-      <c r="H1" s="86"/>
-      <c r="I1" s="86"/>
-      <c r="J1" s="86"/>
-      <c r="K1" s="86"/>
-      <c r="L1" s="86"/>
-      <c r="M1" s="86"/>
-      <c r="N1" s="86"/>
-      <c r="O1" s="86"/>
-      <c r="P1" s="86"/>
-      <c r="Q1" s="86"/>
-      <c r="R1" s="86"/>
-      <c r="S1" s="86"/>
-      <c r="T1" s="86"/>
-      <c r="U1" s="86"/>
-      <c r="V1" s="86"/>
-      <c r="W1" s="86"/>
-      <c r="X1" s="86"/>
-      <c r="Y1" s="86"/>
-      <c r="Z1" s="86"/>
-      <c r="AA1" s="86"/>
-      <c r="AB1" s="86"/>
-      <c r="AC1" s="86"/>
-      <c r="AD1" s="86"/>
-      <c r="AE1" s="86"/>
-      <c r="AF1" s="86"/>
-      <c r="AG1" s="86"/>
-      <c r="AH1" s="86"/>
-      <c r="AI1" s="86"/>
-      <c r="AJ1" s="86"/>
-      <c r="AK1" s="86"/>
-      <c r="AL1" s="86"/>
-      <c r="AM1" s="86"/>
-      <c r="AN1" s="86"/>
-      <c r="AO1" s="86"/>
-      <c r="AP1" s="86"/>
-      <c r="AQ1" s="86"/>
-      <c r="AR1" s="86"/>
-      <c r="AS1" s="89"/>
-      <c r="AT1" s="86"/>
+      <c r="B1" s="70"/>
+      <c r="C1" s="70"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="70"/>
+      <c r="G1" s="70"/>
+      <c r="H1" s="70"/>
+      <c r="I1" s="70"/>
+      <c r="J1" s="70"/>
+      <c r="K1" s="70"/>
+      <c r="L1" s="70"/>
+      <c r="M1" s="70"/>
+      <c r="N1" s="70"/>
+      <c r="O1" s="70"/>
+      <c r="P1" s="70"/>
+      <c r="Q1" s="70"/>
+      <c r="R1" s="70"/>
+      <c r="S1" s="70"/>
+      <c r="T1" s="70"/>
+      <c r="U1" s="70"/>
+      <c r="V1" s="70"/>
+      <c r="W1" s="70"/>
+      <c r="X1" s="70"/>
+      <c r="Y1" s="70"/>
+      <c r="Z1" s="70"/>
+      <c r="AA1" s="70"/>
+      <c r="AB1" s="70"/>
+      <c r="AC1" s="70"/>
+      <c r="AD1" s="70"/>
+      <c r="AE1" s="70"/>
+      <c r="AF1" s="70"/>
+      <c r="AG1" s="70"/>
+      <c r="AH1" s="70"/>
+      <c r="AI1" s="70"/>
+      <c r="AJ1" s="70"/>
+      <c r="AK1" s="70"/>
+      <c r="AL1" s="70"/>
+      <c r="AM1" s="70"/>
+      <c r="AN1" s="70"/>
+      <c r="AO1" s="70"/>
+      <c r="AP1" s="70"/>
+      <c r="AQ1" s="70"/>
+      <c r="AR1" s="70"/>
+      <c r="AS1" s="73"/>
+      <c r="AT1" s="70"/>
     </row>
-    <row r="2" spans="1:46" s="3" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="86" t="s">
+    <row r="2" spans="1:46" s="3" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="70" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="86"/>
-      <c r="C2" s="86"/>
-      <c r="D2" s="87"/>
-      <c r="E2" s="88"/>
-      <c r="F2" s="86"/>
-      <c r="G2" s="86"/>
-      <c r="H2" s="86"/>
-      <c r="I2" s="86"/>
-      <c r="J2" s="86"/>
-      <c r="K2" s="86"/>
-      <c r="L2" s="86"/>
-      <c r="M2" s="86"/>
-      <c r="N2" s="86"/>
-      <c r="O2" s="86"/>
-      <c r="P2" s="86"/>
-      <c r="Q2" s="86"/>
-      <c r="R2" s="86"/>
-      <c r="S2" s="86"/>
-      <c r="T2" s="86"/>
-      <c r="U2" s="86"/>
-      <c r="V2" s="86"/>
-      <c r="W2" s="86"/>
-      <c r="X2" s="86"/>
-      <c r="Y2" s="86"/>
-      <c r="Z2" s="86"/>
-      <c r="AA2" s="86"/>
-      <c r="AB2" s="86"/>
-      <c r="AC2" s="86"/>
-      <c r="AD2" s="86"/>
-      <c r="AE2" s="86"/>
-      <c r="AF2" s="86"/>
-      <c r="AG2" s="86"/>
-      <c r="AH2" s="86"/>
-      <c r="AI2" s="86"/>
-      <c r="AJ2" s="86"/>
-      <c r="AK2" s="86"/>
-      <c r="AL2" s="86"/>
-      <c r="AM2" s="86"/>
-      <c r="AN2" s="86"/>
-      <c r="AO2" s="86"/>
-      <c r="AP2" s="86"/>
-      <c r="AQ2" s="86"/>
-      <c r="AR2" s="86"/>
-      <c r="AS2" s="89"/>
-      <c r="AT2" s="86"/>
+      <c r="B2" s="70"/>
+      <c r="C2" s="70"/>
+      <c r="D2" s="71"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="70"/>
+      <c r="G2" s="70"/>
+      <c r="H2" s="70"/>
+      <c r="I2" s="70"/>
+      <c r="J2" s="70"/>
+      <c r="K2" s="70"/>
+      <c r="L2" s="70"/>
+      <c r="M2" s="70"/>
+      <c r="N2" s="70"/>
+      <c r="O2" s="70"/>
+      <c r="P2" s="70"/>
+      <c r="Q2" s="70"/>
+      <c r="R2" s="70"/>
+      <c r="S2" s="70"/>
+      <c r="T2" s="70"/>
+      <c r="U2" s="70"/>
+      <c r="V2" s="70"/>
+      <c r="W2" s="70"/>
+      <c r="X2" s="70"/>
+      <c r="Y2" s="70"/>
+      <c r="Z2" s="70"/>
+      <c r="AA2" s="70"/>
+      <c r="AB2" s="70"/>
+      <c r="AC2" s="70"/>
+      <c r="AD2" s="70"/>
+      <c r="AE2" s="70"/>
+      <c r="AF2" s="70"/>
+      <c r="AG2" s="70"/>
+      <c r="AH2" s="70"/>
+      <c r="AI2" s="70"/>
+      <c r="AJ2" s="70"/>
+      <c r="AK2" s="70"/>
+      <c r="AL2" s="70"/>
+      <c r="AM2" s="70"/>
+      <c r="AN2" s="70"/>
+      <c r="AO2" s="70"/>
+      <c r="AP2" s="70"/>
+      <c r="AQ2" s="70"/>
+      <c r="AR2" s="70"/>
+      <c r="AS2" s="73"/>
+      <c r="AT2" s="70"/>
     </row>
-    <row r="3" spans="1:46" s="3" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="90" t="s">
+    <row r="3" spans="1:46" s="3" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="74" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="90"/>
-      <c r="C3" s="90"/>
-      <c r="D3" s="91"/>
-      <c r="E3" s="92"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="90"/>
-      <c r="I3" s="90"/>
-      <c r="J3" s="90"/>
-      <c r="K3" s="90"/>
-      <c r="L3" s="90"/>
-      <c r="M3" s="90"/>
-      <c r="N3" s="90"/>
-      <c r="O3" s="90"/>
-      <c r="P3" s="90"/>
-      <c r="Q3" s="90"/>
-      <c r="R3" s="90"/>
-      <c r="S3" s="90"/>
-      <c r="T3" s="90"/>
-      <c r="U3" s="90"/>
-      <c r="V3" s="90"/>
-      <c r="W3" s="90"/>
-      <c r="X3" s="90"/>
-      <c r="Y3" s="90"/>
-      <c r="Z3" s="90"/>
-      <c r="AA3" s="90"/>
-      <c r="AB3" s="90"/>
-      <c r="AC3" s="90"/>
-      <c r="AD3" s="90"/>
-      <c r="AE3" s="90"/>
-      <c r="AF3" s="90"/>
-      <c r="AG3" s="90"/>
-      <c r="AH3" s="90"/>
-      <c r="AI3" s="90"/>
-      <c r="AJ3" s="90"/>
-      <c r="AK3" s="90"/>
-      <c r="AL3" s="90"/>
-      <c r="AM3" s="90"/>
-      <c r="AN3" s="90"/>
-      <c r="AO3" s="90"/>
-      <c r="AP3" s="90"/>
-      <c r="AQ3" s="90"/>
-      <c r="AR3" s="90"/>
-      <c r="AS3" s="93"/>
-      <c r="AT3" s="90"/>
+      <c r="B3" s="74"/>
+      <c r="C3" s="74"/>
+      <c r="D3" s="75"/>
+      <c r="E3" s="76"/>
+      <c r="F3" s="74"/>
+      <c r="G3" s="74"/>
+      <c r="H3" s="74"/>
+      <c r="I3" s="74"/>
+      <c r="J3" s="74"/>
+      <c r="K3" s="74"/>
+      <c r="L3" s="74"/>
+      <c r="M3" s="74"/>
+      <c r="N3" s="74"/>
+      <c r="O3" s="74"/>
+      <c r="P3" s="74"/>
+      <c r="Q3" s="74"/>
+      <c r="R3" s="74"/>
+      <c r="S3" s="74"/>
+      <c r="T3" s="74"/>
+      <c r="U3" s="74"/>
+      <c r="V3" s="74"/>
+      <c r="W3" s="74"/>
+      <c r="X3" s="74"/>
+      <c r="Y3" s="74"/>
+      <c r="Z3" s="74"/>
+      <c r="AA3" s="74"/>
+      <c r="AB3" s="74"/>
+      <c r="AC3" s="74"/>
+      <c r="AD3" s="74"/>
+      <c r="AE3" s="74"/>
+      <c r="AF3" s="74"/>
+      <c r="AG3" s="74"/>
+      <c r="AH3" s="74"/>
+      <c r="AI3" s="74"/>
+      <c r="AJ3" s="74"/>
+      <c r="AK3" s="74"/>
+      <c r="AL3" s="74"/>
+      <c r="AM3" s="74"/>
+      <c r="AN3" s="74"/>
+      <c r="AO3" s="74"/>
+      <c r="AP3" s="74"/>
+      <c r="AQ3" s="74"/>
+      <c r="AR3" s="74"/>
+      <c r="AS3" s="77"/>
+      <c r="AT3" s="74"/>
     </row>
-    <row r="4" spans="1:46" s="3" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:46" s="3" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="4" t="s">
@@ -1937,25 +1691,25 @@
       <c r="AS4" s="2"/>
       <c r="AT4" s="1"/>
     </row>
-    <row r="5" spans="1:46" s="3" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:46" s="3" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
-      <c r="C5" s="87" t="s">
+      <c r="C5" s="71" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="87"/>
-      <c r="E5" s="89"/>
-      <c r="F5" s="87"/>
-      <c r="G5" s="87"/>
-      <c r="H5" s="87"/>
-      <c r="I5" s="87"/>
-      <c r="J5" s="87"/>
-      <c r="K5" s="87"/>
-      <c r="L5" s="87"/>
-      <c r="M5" s="87"/>
-      <c r="N5" s="87"/>
-      <c r="O5" s="87"/>
-      <c r="P5" s="87"/>
+      <c r="D5" s="71"/>
+      <c r="E5" s="73"/>
+      <c r="F5" s="71"/>
+      <c r="G5" s="71"/>
+      <c r="H5" s="71"/>
+      <c r="I5" s="71"/>
+      <c r="J5" s="71"/>
+      <c r="K5" s="71"/>
+      <c r="L5" s="71"/>
+      <c r="M5" s="71"/>
+      <c r="N5" s="71"/>
+      <c r="O5" s="71"/>
+      <c r="P5" s="71"/>
       <c r="Q5" s="11"/>
       <c r="R5" s="11"/>
       <c r="S5" s="12"/>
@@ -1967,18 +1721,18 @@
       <c r="Y5" s="1"/>
       <c r="Z5" s="1"/>
       <c r="AA5" s="1"/>
-      <c r="AB5" s="94" t="s">
+      <c r="AB5" s="78" t="s">
         <v>6</v>
       </c>
-      <c r="AC5" s="94"/>
-      <c r="AD5" s="94"/>
-      <c r="AE5" s="94"/>
-      <c r="AF5" s="94"/>
-      <c r="AG5" s="94"/>
-      <c r="AH5" s="94"/>
-      <c r="AI5" s="94"/>
-      <c r="AJ5" s="94"/>
-      <c r="AK5" s="94"/>
+      <c r="AC5" s="78"/>
+      <c r="AD5" s="78"/>
+      <c r="AE5" s="78"/>
+      <c r="AF5" s="78"/>
+      <c r="AG5" s="78"/>
+      <c r="AH5" s="78"/>
+      <c r="AI5" s="78"/>
+      <c r="AJ5" s="78"/>
+      <c r="AK5" s="78"/>
       <c r="AL5" s="12"/>
       <c r="AM5" s="12"/>
       <c r="AN5" s="12"/>
@@ -1989,25 +1743,25 @@
       <c r="AS5" s="2"/>
       <c r="AT5" s="1"/>
     </row>
-    <row r="6" spans="1:46" s="3" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:46" s="3" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
-      <c r="C6" s="84" t="s">
+      <c r="C6" s="68" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="84"/>
-      <c r="E6" s="85"/>
+      <c r="D6" s="68"/>
+      <c r="E6" s="69"/>
       <c r="F6" s="15"/>
       <c r="G6" s="15"/>
       <c r="H6" s="13"/>
-      <c r="I6" s="84"/>
-      <c r="J6" s="84"/>
-      <c r="K6" s="84"/>
-      <c r="L6" s="84"/>
-      <c r="M6" s="84"/>
-      <c r="N6" s="84"/>
-      <c r="O6" s="84"/>
-      <c r="P6" s="84"/>
+      <c r="I6" s="68"/>
+      <c r="J6" s="68"/>
+      <c r="K6" s="68"/>
+      <c r="L6" s="68"/>
+      <c r="M6" s="68"/>
+      <c r="N6" s="68"/>
+      <c r="O6" s="68"/>
+      <c r="P6" s="68"/>
       <c r="Q6" s="11"/>
       <c r="R6" s="11"/>
       <c r="S6" s="12"/>
@@ -2039,7 +1793,7 @@
       <c r="AS6" s="2"/>
       <c r="AT6" s="1"/>
     </row>
-    <row r="7" spans="1:46" s="3" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:46" s="3" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="16" t="s">
@@ -2089,7 +1843,7 @@
       <c r="AS7" s="2"/>
       <c r="AT7" s="1"/>
     </row>
-    <row r="8" spans="1:46" s="3" customFormat="1" ht="66.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:46" s="3" customFormat="1" ht="66.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="17" t="s">
         <v>9</v>
       </c>
@@ -2229,7 +1983,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:46" s="3" customFormat="1" ht="66.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:46" s="3" customFormat="1" ht="66.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="25"/>
       <c r="B9" s="26"/>
       <c r="C9" s="27"/>
@@ -2281,7 +2035,7 @@
       <c r="AS9" s="29"/>
       <c r="AT9" s="37"/>
     </row>
-    <row r="10" spans="1:46" s="3" customFormat="1" ht="66.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:46" s="3" customFormat="1" ht="66.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="25"/>
       <c r="B10" s="26"/>
       <c r="C10" s="27"/>
@@ -2333,7 +2087,7 @@
       <c r="AS10" s="29"/>
       <c r="AT10" s="37"/>
     </row>
-    <row r="11" spans="1:46" s="3" customFormat="1" ht="66.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:46" s="3" customFormat="1" ht="66.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="25"/>
       <c r="B11" s="26"/>
       <c r="C11" s="27"/>
@@ -2385,7 +2139,7 @@
       <c r="AS11" s="29"/>
       <c r="AT11" s="37"/>
     </row>
-    <row r="12" spans="1:46" s="3" customFormat="1" ht="66.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:46" s="3" customFormat="1" ht="66.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="25"/>
       <c r="B12" s="26"/>
       <c r="C12" s="27"/>
@@ -2437,7 +2191,7 @@
       <c r="AS12" s="29"/>
       <c r="AT12" s="37"/>
     </row>
-    <row r="13" spans="1:46" s="3" customFormat="1" ht="66.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:46" s="3" customFormat="1" ht="66.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="25"/>
       <c r="B13" s="26"/>
       <c r="C13" s="27"/>
@@ -2489,7 +2243,7 @@
       <c r="AS13" s="29"/>
       <c r="AT13" s="37"/>
     </row>
-    <row r="14" spans="1:46" s="3" customFormat="1" ht="66.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:46" s="3" customFormat="1" ht="66.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="25"/>
       <c r="B14" s="26"/>
       <c r="C14" s="27"/>
@@ -2541,7 +2295,7 @@
       <c r="AS14" s="29"/>
       <c r="AT14" s="37"/>
     </row>
-    <row r="15" spans="1:46" s="3" customFormat="1" ht="66.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:46" s="3" customFormat="1" ht="66.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="25"/>
       <c r="B15" s="26"/>
       <c r="C15" s="27"/>
@@ -2601,43 +2355,43 @@
     <mergeCell ref="AB5:AK5"/>
   </mergeCells>
   <conditionalFormatting sqref="B1:B15">
-    <cfRule type="duplicateValues" dxfId="61" priority="6719"/>
-    <cfRule type="duplicateValues" dxfId="60" priority="6715"/>
-    <cfRule type="duplicateValues" dxfId="59" priority="6716"/>
-    <cfRule type="duplicateValues" dxfId="58" priority="6717"/>
-    <cfRule type="duplicateValues" dxfId="57" priority="6718"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="6715"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="6716"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="6717"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="6718"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="6719"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:B1048576">
-    <cfRule type="duplicateValues" dxfId="56" priority="126"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="126"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C15">
-    <cfRule type="duplicateValues" dxfId="55" priority="6732"/>
-    <cfRule type="duplicateValues" dxfId="54" priority="6725"/>
-    <cfRule type="duplicateValues" dxfId="53" priority="6726"/>
-    <cfRule type="duplicateValues" dxfId="52" priority="6727"/>
-    <cfRule type="duplicateValues" dxfId="51" priority="6728"/>
-    <cfRule type="duplicateValues" dxfId="50" priority="6729"/>
-    <cfRule type="duplicateValues" dxfId="49" priority="6730"/>
-    <cfRule type="duplicateValues" dxfId="48" priority="6731"/>
-    <cfRule type="duplicateValues" dxfId="47" priority="6745"/>
-    <cfRule type="duplicateValues" dxfId="46" priority="6733"/>
-    <cfRule type="duplicateValues" dxfId="45" priority="6734"/>
-    <cfRule type="duplicateValues" dxfId="44" priority="6735"/>
-    <cfRule type="duplicateValues" dxfId="43" priority="6736"/>
-    <cfRule type="duplicateValues" dxfId="42" priority="6737"/>
-    <cfRule type="duplicateValues" dxfId="41" priority="6738"/>
-    <cfRule type="duplicateValues" dxfId="40" priority="6739"/>
-    <cfRule type="duplicateValues" dxfId="39" priority="6740"/>
-    <cfRule type="duplicateValues" dxfId="38" priority="6741"/>
-    <cfRule type="duplicateValues" dxfId="37" priority="6742"/>
-    <cfRule type="duplicateValues" dxfId="36" priority="6743"/>
-    <cfRule type="duplicateValues" dxfId="35" priority="6744"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="6725"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="6726"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="6727"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="6728"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="6729"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="6730"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="6731"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="6732"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="6733"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="6734"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="6735"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="6736"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="6737"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="6738"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="6739"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="6740"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="6741"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="6742"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="6743"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="6744"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="6745"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="34" priority="66"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="66"/>
   </conditionalFormatting>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="26" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="28" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter>
     <oddFooter>&amp;L_x000D_&amp;1#&amp;"Aptos"&amp;8&amp;K000000 Sensitivity: LNT Construction Internal Use</oddFooter>
   </headerFooter>
@@ -2649,233 +2403,231 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AE16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="31" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AE32"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="26.25" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.83203125" style="51" customWidth="1"/>
-    <col min="2" max="2" width="38.5" style="75" customWidth="1"/>
-    <col min="3" max="3" width="42.1640625" style="76" customWidth="1"/>
-    <col min="4" max="4" width="45.83203125" style="76" customWidth="1"/>
-    <col min="5" max="5" width="36.6640625" style="76" customWidth="1"/>
-    <col min="6" max="6" width="8.5" style="77" customWidth="1"/>
-    <col min="7" max="7" width="31.83203125" style="51" customWidth="1"/>
-    <col min="8" max="8" width="11.83203125" style="77" customWidth="1"/>
-    <col min="9" max="9" width="28.1640625" style="51" customWidth="1"/>
-    <col min="10" max="10" width="39.6640625" style="78" customWidth="1"/>
-    <col min="11" max="11" width="30.83203125" style="78" customWidth="1"/>
-    <col min="12" max="12" width="18.6640625" style="77" customWidth="1"/>
-    <col min="13" max="13" width="18.33203125" style="51" customWidth="1"/>
-    <col min="14" max="14" width="20.5" style="51" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="6.83203125" style="51" customWidth="1"/>
-    <col min="16" max="16" width="28.33203125" style="51" customWidth="1"/>
-    <col min="17" max="17" width="21.5" style="51" customWidth="1"/>
-    <col min="18" max="18" width="9.1640625" style="51" customWidth="1"/>
-    <col min="19" max="19" width="7.1640625" style="51" customWidth="1"/>
-    <col min="20" max="20" width="27.5" style="51" customWidth="1"/>
-    <col min="21" max="22" width="21.83203125" style="51" customWidth="1"/>
-    <col min="23" max="23" width="19.1640625" style="51" customWidth="1"/>
-    <col min="24" max="25" width="16.83203125" style="51" customWidth="1"/>
-    <col min="26" max="26" width="29" style="51" customWidth="1"/>
-    <col min="27" max="27" width="33.33203125" style="51" customWidth="1"/>
-    <col min="28" max="28" width="19.83203125" style="51" customWidth="1"/>
-    <col min="29" max="29" width="25.1640625" style="51" customWidth="1"/>
-    <col min="30" max="30" width="40.5" style="79" customWidth="1"/>
-    <col min="31" max="31" width="33.5" style="51" customWidth="1"/>
-    <col min="32" max="16384" width="8.6640625" style="80"/>
+    <col min="1" max="1" width="19.42578125" style="46" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="42" style="63" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.42578125" style="64" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="76.85546875" style="64" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.28515625" style="64" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" style="65" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="32.28515625" style="46" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.28515625" style="65" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.42578125" style="46" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.7109375" style="66" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.140625" style="66" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.42578125" style="65" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.140625" style="46" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.7109375" style="46" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.140625" style="46" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="32" style="46" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="23.28515625" style="46" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.85546875" style="46" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.7109375" style="46" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="31.85546875" style="46" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="13" style="46" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="15.85546875" style="46" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.28515625" style="46" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="16.140625" style="46" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="20.140625" style="46" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="28.7109375" style="46" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="26.140625" style="46" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="25.5703125" style="46" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="25.140625" style="46" customWidth="1"/>
+    <col min="30" max="30" width="22.28515625" style="67" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="23.28515625" style="46" bestFit="1" customWidth="1"/>
+    <col min="32" max="16384" width="8.7109375" style="46"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" s="45" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="95" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="95"/>
-      <c r="C1" s="95"/>
-      <c r="D1" s="95"/>
-      <c r="E1" s="95"/>
-      <c r="F1" s="95"/>
-      <c r="G1" s="95"/>
-      <c r="H1" s="95"/>
-      <c r="I1" s="95"/>
-      <c r="J1" s="95"/>
-      <c r="K1" s="95"/>
-      <c r="L1" s="95"/>
-      <c r="M1" s="95"/>
-      <c r="N1" s="95"/>
-      <c r="O1" s="95"/>
-      <c r="P1" s="95"/>
-      <c r="Q1" s="95"/>
-      <c r="R1" s="95"/>
-      <c r="S1" s="95"/>
-      <c r="T1" s="95"/>
-      <c r="U1" s="95"/>
-      <c r="V1" s="95"/>
-      <c r="W1" s="95"/>
-      <c r="X1" s="95"/>
-      <c r="Y1" s="95"/>
-      <c r="Z1" s="95"/>
-      <c r="AA1" s="95"/>
-      <c r="AB1" s="95"/>
-      <c r="AC1" s="95"/>
-      <c r="AD1" s="95"/>
-      <c r="AE1" s="95"/>
+    <row r="1" spans="1:31" x14ac:dyDescent="0.4">
+      <c r="A1" s="79" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="79"/>
+      <c r="C1" s="79"/>
+      <c r="D1" s="79"/>
+      <c r="E1" s="79"/>
+      <c r="F1" s="79"/>
+      <c r="G1" s="79"/>
+      <c r="H1" s="79"/>
+      <c r="I1" s="79"/>
+      <c r="J1" s="79"/>
+      <c r="K1" s="79"/>
+      <c r="L1" s="79"/>
+      <c r="M1" s="79"/>
+      <c r="N1" s="79"/>
+      <c r="O1" s="79"/>
+      <c r="P1" s="79"/>
+      <c r="Q1" s="79"/>
+      <c r="R1" s="79"/>
+      <c r="S1" s="79"/>
+      <c r="T1" s="79"/>
+      <c r="U1" s="79"/>
+      <c r="V1" s="79"/>
+      <c r="W1" s="79"/>
+      <c r="X1" s="79"/>
+      <c r="Y1" s="79"/>
+      <c r="Z1" s="79"/>
+      <c r="AA1" s="79"/>
+      <c r="AB1" s="79"/>
+      <c r="AC1" s="79"/>
+      <c r="AD1" s="79"/>
+      <c r="AE1" s="79"/>
     </row>
-    <row r="2" spans="1:31" s="45" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="95" t="s">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.4">
+      <c r="A2" s="79" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="95"/>
-      <c r="C2" s="95"/>
-      <c r="D2" s="95"/>
-      <c r="E2" s="95"/>
-      <c r="F2" s="95"/>
-      <c r="G2" s="95"/>
-      <c r="H2" s="95"/>
-      <c r="I2" s="95"/>
-      <c r="J2" s="95"/>
-      <c r="K2" s="95"/>
-      <c r="L2" s="95"/>
-      <c r="M2" s="95"/>
-      <c r="N2" s="95"/>
-      <c r="O2" s="95"/>
-      <c r="P2" s="95"/>
-      <c r="Q2" s="95"/>
-      <c r="R2" s="95"/>
-      <c r="S2" s="95"/>
-      <c r="T2" s="95"/>
-      <c r="U2" s="95"/>
-      <c r="V2" s="95"/>
-      <c r="W2" s="95"/>
-      <c r="X2" s="95"/>
-      <c r="Y2" s="95"/>
-      <c r="Z2" s="95"/>
-      <c r="AA2" s="95"/>
-      <c r="AB2" s="95"/>
-      <c r="AC2" s="95"/>
-      <c r="AD2" s="95"/>
-      <c r="AE2" s="95"/>
+      <c r="B2" s="79"/>
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="79"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="79"/>
+      <c r="I2" s="79"/>
+      <c r="J2" s="79"/>
+      <c r="K2" s="79"/>
+      <c r="L2" s="79"/>
+      <c r="M2" s="79"/>
+      <c r="N2" s="79"/>
+      <c r="O2" s="79"/>
+      <c r="P2" s="79"/>
+      <c r="Q2" s="79"/>
+      <c r="R2" s="79"/>
+      <c r="S2" s="79"/>
+      <c r="T2" s="79"/>
+      <c r="U2" s="79"/>
+      <c r="V2" s="79"/>
+      <c r="W2" s="79"/>
+      <c r="X2" s="79"/>
+      <c r="Y2" s="79"/>
+      <c r="Z2" s="79"/>
+      <c r="AA2" s="79"/>
+      <c r="AB2" s="79"/>
+      <c r="AC2" s="79"/>
+      <c r="AD2" s="79"/>
+      <c r="AE2" s="79"/>
     </row>
-    <row r="3" spans="1:31" s="45" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="96" t="s">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.4">
+      <c r="A3" s="80" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="96"/>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="96"/>
-      <c r="L3" s="96"/>
-      <c r="M3" s="96"/>
-      <c r="N3" s="96"/>
-      <c r="O3" s="96"/>
-      <c r="P3" s="96"/>
-      <c r="Q3" s="96"/>
-      <c r="R3" s="96"/>
-      <c r="S3" s="96"/>
-      <c r="T3" s="96"/>
-      <c r="U3" s="96"/>
-      <c r="V3" s="96"/>
-      <c r="W3" s="96"/>
-      <c r="X3" s="96"/>
-      <c r="Y3" s="96"/>
-      <c r="Z3" s="96"/>
-      <c r="AA3" s="96"/>
-      <c r="AB3" s="96"/>
-      <c r="AC3" s="96"/>
-      <c r="AD3" s="96"/>
-      <c r="AE3" s="96"/>
+      <c r="B3" s="80"/>
+      <c r="C3" s="80"/>
+      <c r="D3" s="80"/>
+      <c r="E3" s="80"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="80"/>
+      <c r="H3" s="80"/>
+      <c r="I3" s="80"/>
+      <c r="J3" s="80"/>
+      <c r="K3" s="80"/>
+      <c r="L3" s="80"/>
+      <c r="M3" s="80"/>
+      <c r="N3" s="80"/>
+      <c r="O3" s="80"/>
+      <c r="P3" s="80"/>
+      <c r="Q3" s="80"/>
+      <c r="R3" s="80"/>
+      <c r="S3" s="80"/>
+      <c r="T3" s="80"/>
+      <c r="U3" s="80"/>
+      <c r="V3" s="80"/>
+      <c r="W3" s="80"/>
+      <c r="X3" s="80"/>
+      <c r="Y3" s="80"/>
+      <c r="Z3" s="80"/>
+      <c r="AA3" s="80"/>
+      <c r="AB3" s="80"/>
+      <c r="AC3" s="80"/>
+      <c r="AD3" s="80"/>
+      <c r="AE3" s="80"/>
     </row>
-    <row r="4" spans="1:31" s="45" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="46"/>
-      <c r="B4" s="47"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="48" t="s">
-        <v>38</v>
-      </c>
-      <c r="E4" s="48"/>
-      <c r="F4" s="49"/>
-      <c r="G4" s="48"/>
-      <c r="H4" s="49"/>
-      <c r="I4" s="50"/>
-      <c r="J4" s="47"/>
-      <c r="K4" s="49"/>
-      <c r="L4" s="49"/>
-      <c r="M4" s="48"/>
-      <c r="N4" s="48"/>
-      <c r="O4" s="48"/>
-      <c r="P4" s="48"/>
-      <c r="Q4" s="48"/>
-      <c r="R4" s="46"/>
-      <c r="S4" s="49"/>
-      <c r="T4" s="50"/>
-      <c r="U4" s="50"/>
-      <c r="V4" s="50" t="s">
-        <v>4</v>
-      </c>
-      <c r="W4" s="50"/>
-      <c r="X4" s="50"/>
-      <c r="Y4" s="50"/>
-      <c r="Z4" s="50"/>
-      <c r="AA4" s="51"/>
-      <c r="AB4" s="50"/>
-      <c r="AC4" s="46"/>
-      <c r="AD4" s="48"/>
-      <c r="AE4" s="50"/>
+    <row r="4" spans="1:31" x14ac:dyDescent="0.4">
+      <c r="A4" s="47"/>
+      <c r="B4" s="48"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="49" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="49"/>
+      <c r="F4" s="50"/>
+      <c r="G4" s="49"/>
+      <c r="H4" s="50"/>
+      <c r="I4" s="51"/>
+      <c r="J4" s="48"/>
+      <c r="K4" s="50"/>
+      <c r="L4" s="50"/>
+      <c r="M4" s="49"/>
+      <c r="N4" s="49"/>
+      <c r="O4" s="49"/>
+      <c r="P4" s="49"/>
+      <c r="Q4" s="49"/>
+      <c r="R4" s="47"/>
+      <c r="S4" s="82" t="s">
+        <v>61</v>
+      </c>
+      <c r="T4" s="81"/>
+      <c r="U4" s="81"/>
+      <c r="V4" s="81"/>
+      <c r="W4" s="51"/>
+      <c r="X4" s="51"/>
+      <c r="Y4" s="51"/>
+      <c r="Z4" s="51"/>
+      <c r="AB4" s="51"/>
+      <c r="AC4" s="47"/>
+      <c r="AD4" s="49"/>
+      <c r="AE4" s="51"/>
     </row>
-    <row r="5" spans="1:31" s="45" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="46"/>
-      <c r="B5" s="47"/>
-      <c r="C5" s="46"/>
+    <row r="5" spans="1:31" x14ac:dyDescent="0.4">
+      <c r="A5" s="47"/>
+      <c r="B5" s="48"/>
+      <c r="C5" s="47"/>
       <c r="D5" s="52" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="48"/>
-      <c r="F5" s="49"/>
-      <c r="G5" s="48"/>
-      <c r="H5" s="49"/>
-      <c r="I5" s="49"/>
-      <c r="J5" s="49"/>
-      <c r="K5" s="49"/>
-      <c r="L5" s="49"/>
-      <c r="M5" s="48"/>
-      <c r="N5" s="48"/>
-      <c r="O5" s="48"/>
-      <c r="P5" s="48"/>
-      <c r="Q5" s="48"/>
+      <c r="E5" s="49"/>
+      <c r="F5" s="50"/>
+      <c r="G5" s="49"/>
+      <c r="H5" s="50"/>
+      <c r="I5" s="50"/>
+      <c r="J5" s="50"/>
+      <c r="K5" s="50"/>
+      <c r="L5" s="50"/>
+      <c r="M5" s="49"/>
+      <c r="N5" s="49"/>
+      <c r="O5" s="49"/>
+      <c r="P5" s="49"/>
+      <c r="Q5" s="49"/>
       <c r="R5" s="52"/>
-      <c r="S5" s="53"/>
-      <c r="T5" s="49"/>
-      <c r="U5" s="49"/>
-      <c r="V5" s="48" t="s">
-        <v>6</v>
-      </c>
-      <c r="W5" s="49"/>
-      <c r="X5" s="49"/>
-      <c r="Y5" s="49"/>
-      <c r="Z5" s="49"/>
-      <c r="AA5" s="51"/>
-      <c r="AB5" s="48"/>
-      <c r="AC5" s="49"/>
-      <c r="AD5" s="48"/>
+      <c r="S5" s="81"/>
+      <c r="T5" s="81"/>
+      <c r="U5" s="81"/>
+      <c r="V5" s="81"/>
+      <c r="W5" s="50"/>
+      <c r="X5" s="50"/>
+      <c r="Y5" s="50"/>
+      <c r="Z5" s="50"/>
+      <c r="AB5" s="49"/>
+      <c r="AC5" s="50"/>
+      <c r="AD5" s="49"/>
       <c r="AE5" s="52"/>
     </row>
-    <row r="6" spans="1:31" s="45" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="46"/>
-      <c r="B6" s="47"/>
-      <c r="C6" s="46"/>
+    <row r="6" spans="1:31" x14ac:dyDescent="0.4">
+      <c r="A6" s="47"/>
+      <c r="B6" s="48"/>
+      <c r="C6" s="47"/>
       <c r="D6" s="52" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="E6" s="54"/>
       <c r="F6" s="53"/>
       <c r="G6" s="54"/>
       <c r="H6" s="53"/>
-      <c r="I6" s="49"/>
-      <c r="J6" s="49"/>
+      <c r="I6" s="50"/>
+      <c r="J6" s="50"/>
       <c r="K6" s="53"/>
       <c r="L6" s="53"/>
       <c r="M6" s="54"/>
@@ -2884,26 +2636,26 @@
       <c r="P6" s="54"/>
       <c r="Q6" s="54"/>
       <c r="R6" s="52"/>
-      <c r="S6" s="53"/>
-      <c r="T6" s="49"/>
-      <c r="U6" s="49"/>
-      <c r="V6" s="49"/>
-      <c r="W6" s="49"/>
-      <c r="X6" s="49"/>
-      <c r="Y6" s="49"/>
-      <c r="Z6" s="49"/>
-      <c r="AA6" s="49"/>
-      <c r="AB6" s="49"/>
-      <c r="AC6" s="49"/>
-      <c r="AD6" s="48"/>
-      <c r="AE6" s="49"/>
+      <c r="S6" s="81"/>
+      <c r="T6" s="81"/>
+      <c r="U6" s="81"/>
+      <c r="V6" s="81"/>
+      <c r="W6" s="50"/>
+      <c r="X6" s="50"/>
+      <c r="Y6" s="50"/>
+      <c r="Z6" s="50"/>
+      <c r="AA6" s="50"/>
+      <c r="AB6" s="50"/>
+      <c r="AC6" s="50"/>
+      <c r="AD6" s="49"/>
+      <c r="AE6" s="50"/>
     </row>
-    <row r="7" spans="1:31" s="45" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.4">
       <c r="A7" s="53"/>
       <c r="B7" s="53"/>
       <c r="C7" s="53"/>
       <c r="D7" s="52" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="E7" s="54"/>
       <c r="F7" s="53"/>
@@ -2920,7 +2672,6 @@
       <c r="Q7" s="53"/>
       <c r="R7" s="52"/>
       <c r="S7" s="52"/>
-      <c r="T7" s="51"/>
       <c r="U7" s="52"/>
       <c r="V7" s="52"/>
       <c r="W7" s="52"/>
@@ -2928,12 +2679,12 @@
       <c r="Y7" s="52"/>
       <c r="Z7" s="52"/>
       <c r="AA7" s="52"/>
-      <c r="AB7" s="50"/>
-      <c r="AC7" s="50"/>
+      <c r="AB7" s="51"/>
+      <c r="AC7" s="51"/>
       <c r="AD7" s="54"/>
       <c r="AE7" s="52"/>
     </row>
-    <row r="8" spans="1:31" s="45" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.4">
       <c r="A8" s="53"/>
       <c r="B8" s="53"/>
       <c r="C8" s="53"/>
@@ -2961,852 +2712,168 @@
       <c r="Y8" s="52"/>
       <c r="Z8" s="52"/>
       <c r="AA8" s="52"/>
-      <c r="AB8" s="50"/>
-      <c r="AC8" s="50"/>
+      <c r="AB8" s="51"/>
+      <c r="AC8" s="51"/>
       <c r="AD8" s="54"/>
       <c r="AE8" s="52"/>
     </row>
-    <row r="9" spans="1:31" s="63" customFormat="1" ht="102.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:31" s="45" customFormat="1" ht="52.5" x14ac:dyDescent="0.25">
       <c r="A9" s="59" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="59" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="59" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="59" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="60" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" s="59" t="s">
+        <v>35</v>
+      </c>
+      <c r="G9" s="59" t="s">
+        <v>36</v>
+      </c>
+      <c r="H9" s="59" t="s">
+        <v>37</v>
+      </c>
+      <c r="I9" s="59" t="s">
+        <v>38</v>
+      </c>
+      <c r="J9" s="61" t="s">
+        <v>39</v>
+      </c>
+      <c r="K9" s="61" t="s">
+        <v>40</v>
+      </c>
+      <c r="L9" s="59" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="59" t="s">
+      <c r="M9" s="59" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="59" t="s">
+      <c r="N9" s="59" t="s">
         <v>43</v>
       </c>
-      <c r="D9" s="59" t="s">
+      <c r="O9" s="59" t="s">
         <v>44</v>
       </c>
-      <c r="E9" s="60" t="s">
+      <c r="P9" s="59" t="s">
         <v>45</v>
       </c>
-      <c r="F9" s="59" t="s">
+      <c r="Q9" s="59" t="s">
         <v>46</v>
       </c>
-      <c r="G9" s="59" t="s">
+      <c r="R9" s="59" t="s">
         <v>47</v>
       </c>
-      <c r="H9" s="59" t="s">
+      <c r="S9" s="59" t="s">
         <v>48</v>
       </c>
-      <c r="I9" s="59" t="s">
+      <c r="T9" s="59" t="s">
         <v>49</v>
       </c>
-      <c r="J9" s="61" t="s">
+      <c r="U9" s="59" t="s">
         <v>50</v>
       </c>
-      <c r="K9" s="61" t="s">
+      <c r="V9" s="59" t="s">
         <v>51</v>
       </c>
-      <c r="L9" s="59" t="s">
+      <c r="W9" s="59" t="s">
         <v>52</v>
       </c>
-      <c r="M9" s="59" t="s">
+      <c r="X9" s="59" t="s">
         <v>53</v>
       </c>
-      <c r="N9" s="59" t="s">
+      <c r="Y9" s="59" t="s">
         <v>54</v>
       </c>
-      <c r="O9" s="59" t="s">
+      <c r="Z9" s="59" t="s">
         <v>55</v>
       </c>
-      <c r="P9" s="59" t="s">
+      <c r="AA9" s="59" t="s">
         <v>56</v>
       </c>
-      <c r="Q9" s="59" t="s">
+      <c r="AB9" s="59" t="s">
         <v>57</v>
       </c>
-      <c r="R9" s="59" t="s">
+      <c r="AC9" s="59" t="s">
         <v>58</v>
       </c>
-      <c r="S9" s="59" t="s">
+      <c r="AD9" s="62" t="s">
         <v>59</v>
       </c>
-      <c r="T9" s="59" t="s">
+      <c r="AE9" s="59" t="s">
         <v>60</v>
       </c>
-      <c r="U9" s="59" t="s">
-        <v>61</v>
-      </c>
-      <c r="V9" s="59" t="s">
-        <v>62</v>
-      </c>
-      <c r="W9" s="59" t="s">
-        <v>63</v>
-      </c>
-      <c r="X9" s="59" t="s">
-        <v>64</v>
-      </c>
-      <c r="Y9" s="59" t="s">
-        <v>65</v>
-      </c>
-      <c r="Z9" s="59" t="s">
-        <v>66</v>
-      </c>
-      <c r="AA9" s="59" t="s">
-        <v>67</v>
-      </c>
-      <c r="AB9" s="59" t="s">
-        <v>68</v>
-      </c>
-      <c r="AC9" s="59" t="s">
-        <v>69</v>
-      </c>
-      <c r="AD9" s="62" t="s">
-        <v>70</v>
-      </c>
-      <c r="AE9" s="59" t="s">
-        <v>71</v>
-      </c>
     </row>
-    <row r="10" spans="1:31" s="74" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="64">
-        <v>1</v>
-      </c>
-      <c r="B10" s="65">
-        <v>668659972003</v>
-      </c>
-      <c r="C10" s="65">
-        <v>50398096</v>
-      </c>
-      <c r="D10" s="65" t="s">
-        <v>31</v>
-      </c>
-      <c r="E10" s="66" t="s">
-        <v>74</v>
-      </c>
-      <c r="F10" s="66" t="s">
-        <v>72</v>
-      </c>
-      <c r="G10" s="65" t="s">
-        <v>27</v>
-      </c>
-      <c r="H10" s="81" t="s">
-        <v>80</v>
-      </c>
-      <c r="I10" s="67">
-        <v>46007</v>
-      </c>
-      <c r="J10" s="68">
-        <v>101679392108</v>
-      </c>
-      <c r="K10" s="68">
-        <v>6113277475</v>
-      </c>
-      <c r="L10" s="69">
-        <v>669.04</v>
-      </c>
-      <c r="M10" s="68">
-        <v>14</v>
-      </c>
-      <c r="N10" s="70">
-        <v>0</v>
-      </c>
-      <c r="O10" s="70">
-        <v>0</v>
-      </c>
-      <c r="P10" s="68">
-        <f t="shared" ref="P10:P15" si="0">L10*M10</f>
-        <v>9366.56</v>
-      </c>
-      <c r="Q10" s="71">
-        <f t="shared" ref="Q10:Q15" si="1">L10/4*N10</f>
-        <v>0</v>
-      </c>
-      <c r="R10" s="70">
-        <v>0</v>
-      </c>
-      <c r="S10" s="70">
-        <v>0</v>
-      </c>
-      <c r="T10" s="68">
-        <f t="shared" ref="T10:T15" si="2">SUM(P10:S10)</f>
-        <v>9366.56</v>
-      </c>
-      <c r="U10" s="68">
-        <f t="shared" ref="U10:U15" si="3">IF(P10&gt;15000,1800,P10*12%)</f>
-        <v>1123.9871999999998</v>
-      </c>
-      <c r="V10" s="68">
-        <f t="shared" ref="V10:V15" si="4">T10*0.75%</f>
-        <v>70.249199999999988</v>
-      </c>
-      <c r="W10" s="70">
-        <f t="shared" ref="W10:W15" si="5">IF(T10&gt;10000,200,IF(T10&gt;7500,175,0))</f>
-        <v>175</v>
-      </c>
-      <c r="X10" s="70">
-        <v>25</v>
-      </c>
-      <c r="Y10" s="68">
-        <v>0</v>
-      </c>
-      <c r="Z10" s="68">
-        <f t="shared" ref="Z10:Z15" si="6">SUM(U10:Y10)</f>
-        <v>1394.2363999999998</v>
-      </c>
-      <c r="AA10" s="68">
-        <f t="shared" ref="AA10:AA15" si="7">T10-Z10</f>
-        <v>7972.3235999999997</v>
-      </c>
-      <c r="AB10" s="72"/>
-      <c r="AC10" s="68" t="s">
-        <v>35</v>
-      </c>
-      <c r="AD10" s="65" t="s">
-        <v>36</v>
-      </c>
-      <c r="AE10" s="73"/>
+    <row r="31" spans="17:17" x14ac:dyDescent="0.4">
+      <c r="Q31" s="51"/>
     </row>
-    <row r="11" spans="1:31" s="74" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="64">
-        <f t="shared" ref="A11:A15" si="8">A10+1</f>
-        <v>2</v>
-      </c>
-      <c r="B11" s="65">
-        <v>690783849641</v>
-      </c>
-      <c r="C11" s="65">
-        <v>100425244955</v>
-      </c>
-      <c r="D11" s="65" t="s">
-        <v>29</v>
-      </c>
-      <c r="E11" s="66" t="s">
-        <v>75</v>
-      </c>
-      <c r="F11" s="66" t="s">
-        <v>72</v>
-      </c>
-      <c r="G11" s="65" t="s">
-        <v>26</v>
-      </c>
-      <c r="H11" s="81" t="s">
-        <v>80</v>
-      </c>
-      <c r="I11" s="67">
-        <v>46007</v>
-      </c>
-      <c r="J11" s="68">
-        <v>102235624924</v>
-      </c>
-      <c r="K11" s="68">
-        <v>3417997950</v>
-      </c>
-      <c r="L11" s="69">
-        <v>669.04</v>
-      </c>
-      <c r="M11" s="68">
-        <v>14</v>
-      </c>
-      <c r="N11" s="70">
-        <v>0</v>
-      </c>
-      <c r="O11" s="70">
-        <v>0</v>
-      </c>
-      <c r="P11" s="68">
-        <f t="shared" si="0"/>
-        <v>9366.56</v>
-      </c>
-      <c r="Q11" s="71">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R11" s="70">
-        <v>0</v>
-      </c>
-      <c r="S11" s="70">
-        <v>0</v>
-      </c>
-      <c r="T11" s="68">
-        <f t="shared" si="2"/>
-        <v>9366.56</v>
-      </c>
-      <c r="U11" s="68">
-        <f t="shared" si="3"/>
-        <v>1123.9871999999998</v>
-      </c>
-      <c r="V11" s="68">
-        <f t="shared" si="4"/>
-        <v>70.249199999999988</v>
-      </c>
-      <c r="W11" s="70">
-        <f t="shared" si="5"/>
-        <v>175</v>
-      </c>
-      <c r="X11" s="70">
-        <v>25</v>
-      </c>
-      <c r="Y11" s="68">
-        <v>0</v>
-      </c>
-      <c r="Z11" s="68">
-        <f t="shared" si="6"/>
-        <v>1394.2363999999998</v>
-      </c>
-      <c r="AA11" s="68">
-        <f t="shared" si="7"/>
-        <v>7972.3235999999997</v>
-      </c>
-      <c r="AB11" s="72"/>
-      <c r="AC11" s="68" t="s">
-        <v>35</v>
-      </c>
-      <c r="AD11" s="65" t="s">
-        <v>36</v>
-      </c>
-      <c r="AE11" s="73"/>
-    </row>
-    <row r="12" spans="1:31" s="74" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="64">
-        <f t="shared" si="8"/>
-        <v>3</v>
-      </c>
-      <c r="B12" s="65">
-        <v>621584005209</v>
-      </c>
-      <c r="C12" s="65">
-        <v>103424207342</v>
-      </c>
-      <c r="D12" s="65" t="s">
-        <v>33</v>
-      </c>
-      <c r="E12" s="66" t="s">
-        <v>76</v>
-      </c>
-      <c r="F12" s="66" t="s">
-        <v>72</v>
-      </c>
-      <c r="G12" s="65" t="s">
-        <v>27</v>
-      </c>
-      <c r="H12" s="81" t="s">
-        <v>80</v>
-      </c>
-      <c r="I12" s="67">
-        <v>46007</v>
-      </c>
-      <c r="J12" s="68">
-        <v>101212654335</v>
-      </c>
-      <c r="K12" s="68">
-        <v>3417482237</v>
-      </c>
-      <c r="L12" s="69">
-        <v>669.04</v>
-      </c>
-      <c r="M12" s="68">
-        <v>5</v>
-      </c>
-      <c r="N12" s="70">
-        <v>0</v>
-      </c>
-      <c r="O12" s="70">
-        <v>0</v>
-      </c>
-      <c r="P12" s="68">
-        <f t="shared" si="0"/>
-        <v>3345.2</v>
-      </c>
-      <c r="Q12" s="71">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R12" s="70">
-        <v>0</v>
-      </c>
-      <c r="S12" s="70">
-        <v>0</v>
-      </c>
-      <c r="T12" s="68">
-        <f t="shared" si="2"/>
-        <v>3345.2</v>
-      </c>
-      <c r="U12" s="68">
-        <f t="shared" si="3"/>
-        <v>401.42399999999998</v>
-      </c>
-      <c r="V12" s="68">
-        <f t="shared" si="4"/>
-        <v>25.088999999999999</v>
-      </c>
-      <c r="W12" s="70">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="X12" s="70">
-        <v>25</v>
-      </c>
-      <c r="Y12" s="68">
-        <v>0</v>
-      </c>
-      <c r="Z12" s="68">
-        <f t="shared" si="6"/>
-        <v>451.51299999999998</v>
-      </c>
-      <c r="AA12" s="68">
-        <f t="shared" si="7"/>
-        <v>2893.6869999999999</v>
-      </c>
-      <c r="AB12" s="72"/>
-      <c r="AC12" s="68" t="s">
-        <v>35</v>
-      </c>
-      <c r="AD12" s="65" t="s">
-        <v>36</v>
-      </c>
-      <c r="AE12" s="73"/>
-    </row>
-    <row r="13" spans="1:31" s="74" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="64">
-        <f t="shared" si="8"/>
-        <v>4</v>
-      </c>
-      <c r="B13" s="65">
-        <v>913366880513</v>
-      </c>
-      <c r="C13" s="65">
-        <v>2634723</v>
-      </c>
-      <c r="D13" s="65" t="s">
-        <v>30</v>
-      </c>
-      <c r="E13" s="66" t="s">
-        <v>73</v>
-      </c>
-      <c r="F13" s="66" t="s">
-        <v>72</v>
-      </c>
-      <c r="G13" s="65" t="s">
-        <v>27</v>
-      </c>
-      <c r="H13" s="81" t="s">
-        <v>80</v>
-      </c>
-      <c r="I13" s="67">
-        <v>46011</v>
-      </c>
-      <c r="J13" s="68">
-        <v>101151792159</v>
-      </c>
-      <c r="K13" s="68">
-        <v>3418170810</v>
-      </c>
-      <c r="L13" s="69">
-        <v>669.04</v>
-      </c>
-      <c r="M13" s="68">
-        <v>9</v>
-      </c>
-      <c r="N13" s="70">
-        <v>0</v>
-      </c>
-      <c r="O13" s="70">
-        <v>0</v>
-      </c>
-      <c r="P13" s="68">
-        <f t="shared" si="0"/>
-        <v>6021.36</v>
-      </c>
-      <c r="Q13" s="71">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R13" s="70">
-        <v>0</v>
-      </c>
-      <c r="S13" s="70">
-        <v>0</v>
-      </c>
-      <c r="T13" s="68">
-        <f t="shared" si="2"/>
-        <v>6021.36</v>
-      </c>
-      <c r="U13" s="68">
-        <f t="shared" si="3"/>
-        <v>722.56319999999994</v>
-      </c>
-      <c r="V13" s="68">
-        <f t="shared" si="4"/>
-        <v>45.160199999999996</v>
-      </c>
-      <c r="W13" s="70">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="X13" s="70">
-        <v>25</v>
-      </c>
-      <c r="Y13" s="68">
-        <v>0</v>
-      </c>
-      <c r="Z13" s="68">
-        <f t="shared" si="6"/>
-        <v>792.72339999999997</v>
-      </c>
-      <c r="AA13" s="68">
-        <f t="shared" si="7"/>
-        <v>5228.6365999999998</v>
-      </c>
-      <c r="AB13" s="72"/>
-      <c r="AC13" s="68" t="s">
-        <v>35</v>
-      </c>
-      <c r="AD13" s="65" t="s">
-        <v>36</v>
-      </c>
-      <c r="AE13" s="73"/>
-    </row>
-    <row r="14" spans="1:31" s="74" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="64">
-        <f t="shared" si="8"/>
-        <v>5</v>
-      </c>
-      <c r="B14" s="65">
-        <v>737469683389</v>
-      </c>
-      <c r="C14" s="65">
-        <v>100522079278</v>
-      </c>
-      <c r="D14" s="65" t="s">
-        <v>32</v>
-      </c>
-      <c r="E14" s="66" t="s">
-        <v>77</v>
-      </c>
-      <c r="F14" s="66" t="s">
-        <v>72</v>
-      </c>
-      <c r="G14" s="65" t="s">
-        <v>28</v>
-      </c>
-      <c r="H14" s="81" t="s">
-        <v>79</v>
-      </c>
-      <c r="I14" s="67">
-        <v>46013</v>
-      </c>
-      <c r="J14" s="68">
-        <v>101892561805</v>
-      </c>
-      <c r="K14" s="68">
-        <v>1327480527</v>
-      </c>
-      <c r="L14" s="69">
-        <v>614.41999999999996</v>
-      </c>
-      <c r="M14" s="68">
-        <v>8</v>
-      </c>
-      <c r="N14" s="70">
-        <v>0</v>
-      </c>
-      <c r="O14" s="70">
-        <v>0</v>
-      </c>
-      <c r="P14" s="68">
-        <f t="shared" si="0"/>
-        <v>4915.3599999999997</v>
-      </c>
-      <c r="Q14" s="71">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R14" s="70">
-        <v>0</v>
-      </c>
-      <c r="S14" s="70">
-        <v>0</v>
-      </c>
-      <c r="T14" s="68">
-        <f t="shared" si="2"/>
-        <v>4915.3599999999997</v>
-      </c>
-      <c r="U14" s="68">
-        <f t="shared" si="3"/>
-        <v>589.84319999999991</v>
-      </c>
-      <c r="V14" s="68">
-        <f t="shared" si="4"/>
-        <v>36.865199999999994</v>
-      </c>
-      <c r="W14" s="70">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="X14" s="70">
-        <v>25</v>
-      </c>
-      <c r="Y14" s="68">
-        <v>0</v>
-      </c>
-      <c r="Z14" s="68">
-        <f t="shared" si="6"/>
-        <v>651.70839999999987</v>
-      </c>
-      <c r="AA14" s="68">
-        <f t="shared" si="7"/>
-        <v>4263.6516000000001</v>
-      </c>
-      <c r="AB14" s="72"/>
-      <c r="AC14" s="68" t="s">
-        <v>35</v>
-      </c>
-      <c r="AD14" s="65" t="s">
-        <v>36</v>
-      </c>
-      <c r="AE14" s="73"/>
-    </row>
-    <row r="15" spans="1:31" s="74" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="64">
-        <f t="shared" si="8"/>
-        <v>6</v>
-      </c>
-      <c r="B15" s="65">
-        <v>467928491009</v>
-      </c>
-      <c r="C15" s="65">
-        <v>100522079261</v>
-      </c>
-      <c r="D15" s="65" t="s">
-        <v>34</v>
-      </c>
-      <c r="E15" s="66" t="s">
-        <v>78</v>
-      </c>
-      <c r="F15" s="66" t="s">
-        <v>72</v>
-      </c>
-      <c r="G15" s="65" t="s">
-        <v>28</v>
-      </c>
-      <c r="H15" s="81" t="s">
-        <v>79</v>
-      </c>
-      <c r="I15" s="67">
-        <v>46013</v>
-      </c>
-      <c r="J15" s="68">
-        <v>101892562113</v>
-      </c>
-      <c r="K15" s="68">
-        <v>3418174867</v>
-      </c>
-      <c r="L15" s="69">
-        <v>614.41999999999996</v>
-      </c>
-      <c r="M15" s="68">
-        <v>8</v>
-      </c>
-      <c r="N15" s="70">
-        <v>0</v>
-      </c>
-      <c r="O15" s="70">
-        <v>0</v>
-      </c>
-      <c r="P15" s="68">
-        <f t="shared" si="0"/>
-        <v>4915.3599999999997</v>
-      </c>
-      <c r="Q15" s="71">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R15" s="70">
-        <v>0</v>
-      </c>
-      <c r="S15" s="70">
-        <v>0</v>
-      </c>
-      <c r="T15" s="68">
-        <f t="shared" si="2"/>
-        <v>4915.3599999999997</v>
-      </c>
-      <c r="U15" s="68">
-        <f t="shared" si="3"/>
-        <v>589.84319999999991</v>
-      </c>
-      <c r="V15" s="68">
-        <f t="shared" si="4"/>
-        <v>36.865199999999994</v>
-      </c>
-      <c r="W15" s="70">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="X15" s="70">
-        <v>25</v>
-      </c>
-      <c r="Y15" s="68">
-        <v>0</v>
-      </c>
-      <c r="Z15" s="68">
-        <f t="shared" si="6"/>
-        <v>651.70839999999987</v>
-      </c>
-      <c r="AA15" s="68">
-        <f t="shared" si="7"/>
-        <v>4263.6516000000001</v>
-      </c>
-      <c r="AB15" s="72"/>
-      <c r="AC15" s="68" t="s">
-        <v>35</v>
-      </c>
-      <c r="AD15" s="65" t="s">
-        <v>36</v>
-      </c>
-      <c r="AE15" s="73"/>
-    </row>
-    <row r="16" spans="1:31" s="74" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="64"/>
-      <c r="B16" s="83"/>
-      <c r="C16" s="65"/>
-      <c r="D16" s="65"/>
-      <c r="E16" s="66"/>
-      <c r="F16" s="66"/>
-      <c r="G16" s="65"/>
-      <c r="H16" s="81"/>
-      <c r="I16" s="67"/>
-      <c r="J16" s="68"/>
-      <c r="K16" s="68"/>
-      <c r="L16" s="69"/>
-      <c r="M16" s="82">
-        <f t="shared" ref="M16:AA16" si="9">SUM(M10:M15)</f>
-        <v>58</v>
-      </c>
-      <c r="N16" s="82">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="O16" s="82">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="P16" s="82">
-        <f t="shared" si="9"/>
-        <v>37930.400000000001</v>
-      </c>
-      <c r="Q16" s="82">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="R16" s="82">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="S16" s="82">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="T16" s="82">
-        <f t="shared" si="9"/>
-        <v>37930.400000000001</v>
-      </c>
-      <c r="U16" s="82">
-        <f t="shared" si="9"/>
-        <v>4551.6479999999992</v>
-      </c>
-      <c r="V16" s="82">
-        <f t="shared" si="9"/>
-        <v>284.47799999999995</v>
-      </c>
-      <c r="W16" s="82">
-        <f t="shared" si="9"/>
-        <v>350</v>
-      </c>
-      <c r="X16" s="82">
-        <f t="shared" si="9"/>
-        <v>150</v>
-      </c>
-      <c r="Y16" s="82">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="Z16" s="82">
-        <f t="shared" si="9"/>
-        <v>5336.1259999999984</v>
-      </c>
-      <c r="AA16" s="82">
-        <f t="shared" si="9"/>
-        <v>32594.273999999998</v>
-      </c>
-      <c r="AB16" s="72"/>
-      <c r="AC16" s="68"/>
-      <c r="AD16" s="65"/>
-      <c r="AE16" s="73"/>
+    <row r="32" spans="17:17" x14ac:dyDescent="0.4">
+      <c r="Q32" s="49"/>
     </row>
   </sheetData>
   <autoFilter ref="A9:AE9" xr:uid="{BDC202CF-CAC5-4C7F-AF81-A4D2D85B9E48}"/>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:AE1"/>
     <mergeCell ref="A2:AE2"/>
     <mergeCell ref="A3:AE3"/>
+    <mergeCell ref="S4:V6"/>
   </mergeCells>
-  <conditionalFormatting sqref="B1:B15">
-    <cfRule type="duplicateValues" dxfId="33" priority="6662"/>
-    <cfRule type="duplicateValues" dxfId="32" priority="6663"/>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B1:B1048576">
-    <cfRule type="duplicateValues" dxfId="31" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B4:B9">
-    <cfRule type="duplicateValues" dxfId="30" priority="182"/>
-    <cfRule type="duplicateValues" dxfId="29" priority="181"/>
-    <cfRule type="duplicateValues" dxfId="28" priority="180"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B16">
-    <cfRule type="duplicateValues" dxfId="27" priority="6467"/>
-    <cfRule type="duplicateValues" dxfId="26" priority="6462"/>
-    <cfRule type="duplicateValues" dxfId="25" priority="6466"/>
-    <cfRule type="duplicateValues" dxfId="24" priority="6465"/>
-    <cfRule type="duplicateValues" dxfId="23" priority="6464"/>
-    <cfRule type="duplicateValues" dxfId="22" priority="6463"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="180"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="181"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="182"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C9">
     <cfRule type="duplicateValues" dxfId="21" priority="179"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C1:C16">
-    <cfRule type="duplicateValues" dxfId="20" priority="6668"/>
-    <cfRule type="duplicateValues" dxfId="19" priority="6667"/>
-    <cfRule type="duplicateValues" dxfId="18" priority="6666"/>
-    <cfRule type="duplicateValues" dxfId="17" priority="6669"/>
-  </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="16" priority="174"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="174"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:C9">
-    <cfRule type="duplicateValues" dxfId="15" priority="172"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="173"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="172"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="173"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:J1048576">
-    <cfRule type="duplicateValues" dxfId="13" priority="6659"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="6659"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1:K9">
-    <cfRule type="duplicateValues" dxfId="12" priority="6445"/>
-    <cfRule type="duplicateValues" dxfId="11" priority="6443"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="149"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="6444"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="149"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="6443"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="6444"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="6445"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4:K9">
-    <cfRule type="duplicateValues" dxfId="8" priority="6451"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="6452"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="6446"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="6450"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="6449"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="6448"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="6447"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="6446"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="6447"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="6448"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="6449"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="6450"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="6451"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="6452"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K10:K15">
-    <cfRule type="duplicateValues" dxfId="1" priority="6674"/>
+  <conditionalFormatting sqref="B1:B9">
+    <cfRule type="duplicateValues" dxfId="5" priority="6746"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="6747"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K16">
-    <cfRule type="duplicateValues" dxfId="0" priority="6566"/>
+  <conditionalFormatting sqref="C1:C9">
+    <cfRule type="duplicateValues" dxfId="3" priority="6751"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="6752"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="6753"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="6754"/>
   </conditionalFormatting>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="17" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="19" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter>
     <oddFooter>&amp;L_x000D_&amp;1#&amp;"Calibri"&amp;8&amp;K000000 Sensitivity: LNT Construction Internal Use</oddFooter>
   </headerFooter>

</xml_diff>